<commit_message>
feat: atualização dos escudos dos times
</commit_message>
<xml_diff>
--- a/public/team-names.xlsx
+++ b/public/team-names.xlsx
@@ -1,19 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dna-futsal\dna_frontend\public\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67ED4BF0-D41D-4605-B980-DDC296FD8CA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="INICIAÇÃO A1" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="BASE A1" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="INICIAÇÃO A2" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="BASE A2" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="INICIAÇÃO A3" sheetId="5" r:id="rId9"/>
-    <sheet state="visible" name="BASE A3" sheetId="6" r:id="rId10"/>
+    <sheet name="INICIAÇÃO A1" sheetId="1" r:id="rId1"/>
+    <sheet name="BASE A1" sheetId="2" r:id="rId2"/>
+    <sheet name="INICIAÇÃO A2" sheetId="3" r:id="rId3"/>
+    <sheet name="BASE A2" sheetId="4" r:id="rId4"/>
+    <sheet name="INICIAÇÃO A3" sheetId="5" r:id="rId5"/>
+    <sheet name="BASE A3" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">'INICIAÇÃO A2'!$A$2:$D$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'INICIAÇÃO A2'!$A$2:$D$26</definedName>
   </definedNames>
-  <calcPr/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -929,62 +950,70 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="10">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="Oswald"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -995,7 +1024,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1011,99 +1040,64 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+  <cellXfs count="13">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" wrapText="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1111,7 +1105,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1301,1033 +1295,1028 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:D28"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="62.5"/>
-    <col customWidth="1" min="2" max="2" width="17.13"/>
-    <col customWidth="1" min="4" max="4" width="24.63"/>
+    <col min="1" max="1" width="62.42578125" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="4" max="4" width="24.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.0" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+    </row>
+    <row r="2" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="8" t="s">
+      <c r="C3" s="4"/>
+      <c r="D3" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="8" t="s">
+      <c r="C4" s="4"/>
+      <c r="D4" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="8" t="s">
+      <c r="C5" s="4"/>
+      <c r="D5" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="6"/>
-      <c r="D6" s="8" t="s">
+      <c r="C6" s="4"/>
+      <c r="D6" s="5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="8" t="s">
+      <c r="C7" s="4"/>
+      <c r="D7" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="s">
+    <row r="8" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="8" t="s">
+      <c r="C8" s="4"/>
+      <c r="D8" s="5" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="6"/>
-      <c r="D9" s="8" t="s">
+      <c r="C9" s="4"/>
+      <c r="D9" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="8" t="s">
+      <c r="C10" s="4"/>
+      <c r="D10" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="8" t="s">
+      <c r="C11" s="4"/>
+      <c r="D11" s="5" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="8" t="s">
+      <c r="C12" s="4"/>
+      <c r="D12" s="5" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="8" t="s">
+      <c r="C13" s="4"/>
+      <c r="D13" s="5" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="s">
+    <row r="14" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="15" t="s">
+      <c r="C14" s="4"/>
+      <c r="D14" s="10" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="s">
+    <row r="15" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="9" t="s">
+      <c r="C15" s="4"/>
+      <c r="D15" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="s">
+    <row r="16" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="15" t="s">
+      <c r="C16" s="4"/>
+      <c r="D16" s="10" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="s">
+    <row r="17" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="C17" s="6"/>
-      <c r="D17" s="9" t="s">
+      <c r="C17" s="4"/>
+      <c r="D17" s="6" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="s">
+    <row r="18" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="C18" s="6"/>
-      <c r="D18" s="15" t="s">
+      <c r="C18" s="4"/>
+      <c r="D18" s="10" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="s">
+    <row r="19" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="C19" s="6"/>
-      <c r="D19" s="8" t="s">
+      <c r="C19" s="4"/>
+      <c r="D19" s="5" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="s">
+    <row r="20" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="C20" s="6"/>
-      <c r="D20" s="8" t="s">
+      <c r="C20" s="4"/>
+      <c r="D20" s="5" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="s">
+    <row r="21" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="C21" s="6"/>
-      <c r="D21" s="8" t="s">
+      <c r="C21" s="4"/>
+      <c r="D21" s="5" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="s">
+    <row r="22" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C22" s="6"/>
-      <c r="D22" s="8" t="s">
+      <c r="C22" s="4"/>
+      <c r="D22" s="5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="s">
+    <row r="23" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="6"/>
-      <c r="D23" s="9" t="s">
+      <c r="C23" s="4"/>
+      <c r="D23" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="s">
+    <row r="24" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="8" t="s">
+      <c r="C24" s="4"/>
+      <c r="D24" s="5" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="s">
+    <row r="25" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="C25" s="6"/>
-      <c r="D25" s="15" t="s">
+      <c r="C25" s="4"/>
+      <c r="D25" s="10" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="s">
+    <row r="26" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="C26" s="6"/>
-      <c r="D26" s="15" t="s">
+      <c r="C26" s="4"/>
+      <c r="D26" s="10" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="17"/>
-    </row>
-    <row r="28">
-      <c r="D28" s="18"/>
+    <row r="27" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+    </row>
+    <row r="28" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="D28" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="D3"/>
-    <hyperlink r:id="rId2" ref="D4"/>
-    <hyperlink r:id="rId3" ref="D5"/>
-    <hyperlink r:id="rId4" ref="D6"/>
-    <hyperlink r:id="rId5" ref="D7"/>
-    <hyperlink r:id="rId6" ref="D8"/>
-    <hyperlink r:id="rId7" ref="D9"/>
-    <hyperlink r:id="rId8" ref="D10"/>
-    <hyperlink r:id="rId9" ref="D11"/>
-    <hyperlink r:id="rId10" ref="D12"/>
-    <hyperlink r:id="rId11" ref="D13"/>
-    <hyperlink r:id="rId12" ref="D14"/>
-    <hyperlink r:id="rId13" ref="D15"/>
-    <hyperlink r:id="rId14" ref="D16"/>
-    <hyperlink r:id="rId15" ref="D17"/>
-    <hyperlink r:id="rId16" ref="D18"/>
-    <hyperlink r:id="rId17" ref="D19"/>
-    <hyperlink r:id="rId18" ref="D20"/>
-    <hyperlink r:id="rId19" ref="D21"/>
-    <hyperlink r:id="rId20" ref="D22"/>
-    <hyperlink r:id="rId21" ref="D23"/>
-    <hyperlink r:id="rId22" ref="D24"/>
-    <hyperlink r:id="rId23" ref="D25"/>
-    <hyperlink r:id="rId24" ref="D26"/>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="D5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="D6" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="D7" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="D8" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="D9" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="D10" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="D11" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="D12" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="D13" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="D14" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="D15" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="D16" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="D17" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="D18" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="D19" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="D20" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="D21" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="D22" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="D23" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="D24" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="D25" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="D26" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
   </hyperlinks>
-  <drawing r:id="rId25"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:D27"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="62.5"/>
-    <col customWidth="1" min="2" max="2" width="18.75"/>
-    <col customWidth="1" min="3" max="3" width="22.13"/>
+    <col min="1" max="1" width="62.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" customWidth="1"/>
+    <col min="4" max="4" width="28.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.0" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="11" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+    </row>
+    <row r="2" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="5" t="str">
+      <c r="B3" s="4" t="str">
         <f>VLOOKUP(A3, 'INICIAÇÃO A1'!$A$1:$D$26, 2, FALSE)</f>
         <v>PALMEIRAS</v>
       </c>
-      <c r="C3" s="8" t="str">
+      <c r="D3" s="5" t="str">
         <f>VLOOKUP(A3, 'INICIAÇÃO A1'!$A$1:$D$26, 4, FALSE)</f>
         <v>Palmeiras_logo.svg.png</v>
       </c>
-      <c r="D3" s="6"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="s">
+    </row>
+    <row r="4" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B4" s="5" t="str">
+      <c r="B4" s="4" t="str">
         <f>VLOOKUP(A4, 'INICIAÇÃO A1'!$A$1:$D$26, 2, FALSE)</f>
         <v>SANTOS</v>
       </c>
-      <c r="C4" s="12" t="str">
+      <c r="D4" s="9" t="str">
         <f>VLOOKUP(A4, 'INICIAÇÃO A1'!$A$1:$D$26, 4, FALSE)</f>
         <v>Santos_Logo.png</v>
       </c>
-      <c r="D4" s="6"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="s">
+    </row>
+    <row r="5" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="5" t="str">
+      <c r="B5" s="4" t="str">
         <f>VLOOKUP(A5, 'INICIAÇÃO A1'!$A$1:$D$26, 2, FALSE)</f>
         <v>SÃO PAULO</v>
       </c>
-      <c r="C5" s="8" t="str">
+      <c r="D5" s="5" t="str">
         <f>VLOOKUP(A5, 'INICIAÇÃO A1'!$A$1:$D$26, 4, FALSE)</f>
         <v>São_Paulo.png</v>
       </c>
-      <c r="D5" s="6"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="s">
+    </row>
+    <row r="6" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="D6" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D6" s="6"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="s">
+    </row>
+    <row r="7" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B7" s="5" t="str">
+      <c r="B7" s="4" t="str">
         <f>VLOOKUP(A7, 'INICIAÇÃO A1'!$A$1:$D$26, 2, FALSE)</f>
         <v>LAUSANNE</v>
       </c>
-      <c r="C7" s="12" t="str">
+      <c r="D7" s="9" t="str">
         <f>VLOOKUP(A7, 'INICIAÇÃO A1'!$A$1:$D$26, 4, FALSE)</f>
         <v>Lausanne_Paulista.png</v>
       </c>
-      <c r="D7" s="6"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="s">
+    </row>
+    <row r="8" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B8" s="5" t="str">
+      <c r="B8" s="4" t="str">
         <f>VLOOKUP(A8, 'INICIAÇÃO A1'!$A$1:$D$26, 2, FALSE)</f>
         <v>SÃO CAETANO</v>
       </c>
-      <c r="C8" s="12" t="str">
+      <c r="D8" s="9" t="str">
         <f>VLOOKUP(A8, 'INICIAÇÃO A1'!$A$1:$D$26, 4, FALSE)</f>
         <v>RS_São_Caetano.png</v>
       </c>
-      <c r="D8" s="6"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="s">
+    </row>
+    <row r="9" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B9" s="5" t="str">
+      <c r="B9" s="4" t="str">
         <f>VLOOKUP(A9, 'INICIAÇÃO A1'!$A$1:$D$26, 2, FALSE)</f>
         <v>LIGA SÃO CAETANO</v>
       </c>
-      <c r="C9" s="12" t="str">
+      <c r="D9" s="9" t="str">
         <f>VLOOKUP(A9, 'INICIAÇÃO A1'!$A$1:$D$26, 4, FALSE)</f>
         <v>Liga Sao Caetano.jpg</v>
       </c>
-      <c r="D9" s="6"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="s">
+    </row>
+    <row r="10" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="5" t="str">
+      <c r="B10" s="4" t="str">
         <f>VLOOKUP(A10, 'INICIAÇÃO A1'!$A$1:$D$26, 2, FALSE)</f>
         <v>ASF / MAGNUS</v>
       </c>
-      <c r="C10" s="12" t="str">
+      <c r="D10" s="9" t="str">
         <f>VLOOKUP(A10, 'INICIAÇÃO A1'!$A$1:$D$26, 4, FALSE)</f>
         <v>ASF_Magnus.png</v>
       </c>
-      <c r="D10" s="6"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="s">
+    </row>
+    <row r="11" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="5" t="str">
+      <c r="B11" s="4" t="str">
         <f>VLOOKUP(A11, 'INICIAÇÃO A1'!$A$1:$D$26, 2, FALSE)</f>
         <v>CORINTHIANS</v>
       </c>
-      <c r="C11" s="8" t="str">
+      <c r="D11" s="5" t="str">
         <f>VLOOKUP(A11, 'INICIAÇÃO A1'!$A$1:$D$26, 4, FALSE)</f>
         <v>Corinthians_logo.png</v>
       </c>
-      <c r="D11" s="6"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="s">
+    </row>
+    <row r="12" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B12" s="5" t="str">
+      <c r="B12" s="4" t="str">
         <f>VLOOKUP(A12, 'INICIAÇÃO A1'!$A$1:$D$26, 2, FALSE)</f>
         <v>JUVENTUS</v>
       </c>
-      <c r="C12" s="12" t="str">
+      <c r="D12" s="9" t="str">
         <f>VLOOKUP(A12, 'INICIAÇÃO A1'!$A$1:$D$26, 4, FALSE)</f>
         <v>CA_Juventus_logo.svg.png</v>
       </c>
-      <c r="D12" s="6"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="s">
+    </row>
+    <row r="13" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="D13" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="D13" s="6"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="s">
+    </row>
+    <row r="14" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B14" s="5" t="str">
+      <c r="B14" s="4" t="str">
         <f>VLOOKUP(A14, 'INICIAÇÃO A1'!$A$1:$D$26, 2, FALSE)</f>
         <v>AUDAX</v>
       </c>
-      <c r="C14" s="12" t="str">
+      <c r="D14" s="9" t="str">
         <f>VLOOKUP(A14, 'INICIAÇÃO A1'!$A$1:$D$26, 4, FALSE)</f>
         <v>Audax_Osasco.png</v>
       </c>
-      <c r="D14" s="6"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="s">
+    </row>
+    <row r="15" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="D15" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="D15" s="6"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="s">
+    </row>
+    <row r="16" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="D16" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="D16" s="6"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="s">
+    </row>
+    <row r="17" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="D17" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="D17" s="6"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="s">
+    </row>
+    <row r="18" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="D18" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="D18" s="6"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="s">
+    </row>
+    <row r="19" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C19" s="16" t="s">
+      <c r="D19" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="D19" s="6"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="s">
+    </row>
+    <row r="20" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="D20" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="D20" s="6"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="s">
+    </row>
+    <row r="21" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="C21" s="16" t="s">
+      <c r="D21" s="10" t="s">
         <v>191</v>
       </c>
-      <c r="D21" s="6"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="s">
+    </row>
+    <row r="22" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C22" s="12" t="str">
+      <c r="D22" s="9" t="str">
         <f>VLOOKUP(A22, 'INICIAÇÃO A1'!$A$1:$D$26, 4, FALSE)</f>
         <v>AD_Indaiatuba.png</v>
       </c>
-      <c r="D22" s="6"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="5"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="5"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="5"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="5"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
+    </row>
+    <row r="23" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+    </row>
+    <row r="24" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+    </row>
+    <row r="25" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+    </row>
+    <row r="26" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+    </row>
+    <row r="27" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="C6"/>
-    <hyperlink r:id="rId2" ref="C13"/>
-    <hyperlink r:id="rId3" ref="C15"/>
-    <hyperlink r:id="rId4" ref="C16"/>
-    <hyperlink r:id="rId5" ref="C17"/>
-    <hyperlink r:id="rId6" ref="C18"/>
-    <hyperlink r:id="rId7" ref="C19"/>
-    <hyperlink r:id="rId8" ref="C20"/>
-    <hyperlink r:id="rId9" ref="C21"/>
+    <hyperlink ref="D6" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="D13" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="D15" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="D16" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="D17" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
+    <hyperlink ref="D18" r:id="rId6" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
+    <hyperlink ref="D19" r:id="rId7" xr:uid="{00000000-0004-0000-0100-000006000000}"/>
+    <hyperlink ref="D20" r:id="rId8" xr:uid="{00000000-0004-0000-0100-000007000000}"/>
+    <hyperlink ref="D21" r:id="rId9" xr:uid="{00000000-0004-0000-0100-000008000000}"/>
   </hyperlinks>
-  <drawing r:id="rId10"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:D27"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="62.5"/>
-    <col customWidth="1" min="2" max="2" width="17.13"/>
-    <col customWidth="1" min="4" max="4" width="19.63"/>
+    <col min="1" max="1" width="62.42578125" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="4" max="4" width="19.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.0" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="11" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+    </row>
+    <row r="2" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="10" t="s">
+      <c r="C3" s="4"/>
+      <c r="D3" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="11" t="s">
+      <c r="C4" s="4"/>
+      <c r="D4" s="8" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="10" t="s">
+      <c r="C5" s="4"/>
+      <c r="D5" s="7" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="6"/>
-      <c r="D6" s="10" t="s">
+      <c r="C6" s="4"/>
+      <c r="D6" s="7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="10" t="s">
+      <c r="C7" s="4"/>
+      <c r="D7" s="7" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="s">
+    <row r="8" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="11" t="s">
+      <c r="C8" s="4"/>
+      <c r="D8" s="8" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C9" s="6"/>
-      <c r="D9" s="11" t="s">
+      <c r="C9" s="4"/>
+      <c r="D9" s="8" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="10" t="s">
+      <c r="C10" s="4"/>
+      <c r="D10" s="7" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="16" t="s">
+      <c r="C11" s="4"/>
+      <c r="D11" s="10" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="10" t="s">
+      <c r="C12" s="4"/>
+      <c r="D12" s="7" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="10" t="s">
+      <c r="C13" s="4"/>
+      <c r="D13" s="7" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="s">
+    <row r="14" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="10" t="s">
+      <c r="C14" s="4"/>
+      <c r="D14" s="7" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="s">
+    <row r="15" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="10" t="s">
+      <c r="C15" s="4"/>
+      <c r="D15" s="7" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="s">
+    <row r="16" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="10" t="s">
+      <c r="C16" s="4"/>
+      <c r="D16" s="7" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="s">
+    <row r="17" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="C17" s="6"/>
-      <c r="D17" s="11" t="s">
+      <c r="C17" s="4"/>
+      <c r="D17" s="8" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="s">
+    <row r="18" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C18" s="6"/>
-      <c r="D18" s="11" t="s">
+      <c r="C18" s="4"/>
+      <c r="D18" s="8" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="s">
+    <row r="19" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="C19" s="6"/>
-      <c r="D19" s="10" t="s">
+      <c r="C19" s="4"/>
+      <c r="D19" s="7" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="s">
+    <row r="20" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C20" s="6"/>
-      <c r="D20" s="10" t="s">
+      <c r="C20" s="4"/>
+      <c r="D20" s="7" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="s">
+    <row r="21" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="C21" s="6"/>
-      <c r="D21" s="10" t="s">
+      <c r="C21" s="4"/>
+      <c r="D21" s="7" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="s">
+    <row r="22" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="C22" s="6"/>
-      <c r="D22" s="10" t="s">
+      <c r="C22" s="4"/>
+      <c r="D22" s="7" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="s">
+    <row r="23" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="C23" s="6"/>
-      <c r="D23" s="11" t="s">
+      <c r="C23" s="4"/>
+      <c r="D23" s="8" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="s">
+    <row r="24" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="10" t="s">
+      <c r="C24" s="4"/>
+      <c r="D24" s="7" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="s">
+    <row r="25" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="C25" s="6"/>
-      <c r="D25" s="10" t="s">
+      <c r="C25" s="4"/>
+      <c r="D25" s="7" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="s">
+    <row r="26" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="4" t="s">
         <v>259</v>
       </c>
-      <c r="C26" s="6"/>
-      <c r="D26" s="11" t="s">
+      <c r="C26" s="4"/>
+      <c r="D26" s="8" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
+    <row r="27" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="$A$2:$D$26">
-    <sortState ref="A2:D26">
+  <autoFilter ref="A2:D26" xr:uid="{00000000-0009-0000-0000-000002000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D26">
       <sortCondition ref="A2:A26"/>
     </sortState>
   </autoFilter>
@@ -2335,666 +2324,674 @@
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="D3"/>
-    <hyperlink r:id="rId2" ref="D4"/>
-    <hyperlink r:id="rId3" ref="D5"/>
-    <hyperlink r:id="rId4" ref="D6"/>
-    <hyperlink r:id="rId5" ref="D7"/>
-    <hyperlink r:id="rId6" ref="D8"/>
-    <hyperlink r:id="rId7" ref="D9"/>
-    <hyperlink r:id="rId8" ref="D10"/>
-    <hyperlink r:id="rId9" ref="D11"/>
-    <hyperlink r:id="rId10" ref="D12"/>
-    <hyperlink r:id="rId11" ref="D13"/>
-    <hyperlink r:id="rId12" ref="D14"/>
-    <hyperlink r:id="rId13" ref="D15"/>
-    <hyperlink r:id="rId14" ref="D16"/>
-    <hyperlink r:id="rId15" ref="D17"/>
-    <hyperlink r:id="rId16" ref="D18"/>
-    <hyperlink r:id="rId17" ref="D19"/>
-    <hyperlink r:id="rId18" ref="D20"/>
-    <hyperlink r:id="rId19" ref="D21"/>
-    <hyperlink r:id="rId20" ref="D22"/>
-    <hyperlink r:id="rId21" ref="D23"/>
-    <hyperlink r:id="rId22" ref="D24"/>
-    <hyperlink r:id="rId23" ref="D25"/>
-    <hyperlink r:id="rId24" ref="D26"/>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
+    <hyperlink ref="D4" r:id="rId2" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
+    <hyperlink ref="D5" r:id="rId3" xr:uid="{00000000-0004-0000-0200-000002000000}"/>
+    <hyperlink ref="D6" r:id="rId4" xr:uid="{00000000-0004-0000-0200-000003000000}"/>
+    <hyperlink ref="D7" r:id="rId5" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
+    <hyperlink ref="D8" r:id="rId6" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
+    <hyperlink ref="D9" r:id="rId7" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
+    <hyperlink ref="D10" r:id="rId8" xr:uid="{00000000-0004-0000-0200-000007000000}"/>
+    <hyperlink ref="D11" r:id="rId9" xr:uid="{00000000-0004-0000-0200-000008000000}"/>
+    <hyperlink ref="D12" r:id="rId10" xr:uid="{00000000-0004-0000-0200-000009000000}"/>
+    <hyperlink ref="D13" r:id="rId11" xr:uid="{00000000-0004-0000-0200-00000A000000}"/>
+    <hyperlink ref="D14" r:id="rId12" xr:uid="{00000000-0004-0000-0200-00000B000000}"/>
+    <hyperlink ref="D15" r:id="rId13" xr:uid="{00000000-0004-0000-0200-00000C000000}"/>
+    <hyperlink ref="D16" r:id="rId14" xr:uid="{00000000-0004-0000-0200-00000D000000}"/>
+    <hyperlink ref="D17" r:id="rId15" xr:uid="{00000000-0004-0000-0200-00000E000000}"/>
+    <hyperlink ref="D18" r:id="rId16" xr:uid="{00000000-0004-0000-0200-00000F000000}"/>
+    <hyperlink ref="D19" r:id="rId17" xr:uid="{00000000-0004-0000-0200-000010000000}"/>
+    <hyperlink ref="D20" r:id="rId18" xr:uid="{00000000-0004-0000-0200-000011000000}"/>
+    <hyperlink ref="D21" r:id="rId19" xr:uid="{00000000-0004-0000-0200-000012000000}"/>
+    <hyperlink ref="D22" r:id="rId20" xr:uid="{00000000-0004-0000-0200-000013000000}"/>
+    <hyperlink ref="D23" r:id="rId21" xr:uid="{00000000-0004-0000-0200-000014000000}"/>
+    <hyperlink ref="D24" r:id="rId22" xr:uid="{00000000-0004-0000-0200-000015000000}"/>
+    <hyperlink ref="D25" r:id="rId23" xr:uid="{00000000-0004-0000-0200-000016000000}"/>
+    <hyperlink ref="D26" r:id="rId24" xr:uid="{00000000-0004-0000-0200-000017000000}"/>
   </hyperlinks>
-  <drawing r:id="rId25"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:D27"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="62.5"/>
-    <col customWidth="1" min="2" max="2" width="17.13"/>
-    <col customWidth="1" min="3" max="3" width="23.0"/>
-    <col customWidth="1" min="4" max="4" width="28.5"/>
+    <col min="1" max="1" width="62.42578125" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="3" max="3" width="23" customWidth="1"/>
+    <col min="4" max="4" width="28.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.0" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+    </row>
+    <row r="2" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="9" t="s">
+      <c r="C3" s="4"/>
+      <c r="D3" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="10" t="s">
+      <c r="C4" s="4"/>
+      <c r="D4" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="10" t="s">
+      <c r="C5" s="4"/>
+      <c r="D5" s="7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="10" t="s">
+      <c r="C6" s="4"/>
+      <c r="D6" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="9" t="s">
+      <c r="C7" s="4"/>
+      <c r="D7" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="s">
+    <row r="8" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="13"/>
-      <c r="D8" s="8" t="s">
+      <c r="C8" s="4"/>
+      <c r="D8" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C9" s="13"/>
-      <c r="D9" s="8" t="s">
+      <c r="C9" s="4"/>
+      <c r="D9" s="5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="10" t="s">
+      <c r="C10" s="4"/>
+      <c r="D10" s="7" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="14"/>
-      <c r="D11" s="11" t="s">
+      <c r="C11" s="4"/>
+      <c r="D11" s="8" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="10" t="s">
+      <c r="C12" s="4"/>
+      <c r="D12" s="7" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="11" t="s">
+      <c r="C13" s="4"/>
+      <c r="D13" s="8" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="s">
+    <row r="14" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15" t="s">
+      <c r="C14" s="10"/>
+      <c r="D14" s="10" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="s">
+    <row r="15" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="8" t="s">
+      <c r="C15" s="4"/>
+      <c r="D15" s="5" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="s">
+    <row r="16" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="10" t="s">
+      <c r="C16" s="4"/>
+      <c r="D16" s="7" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="s">
+    <row r="17" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="C17" s="6"/>
-      <c r="D17" s="10" t="s">
+      <c r="C17" s="4"/>
+      <c r="D17" s="7" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="s">
+    <row r="18" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="s">
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+    </row>
+    <row r="19" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="s">
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+    </row>
+    <row r="20" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="s">
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+    </row>
+    <row r="21" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="s">
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+    </row>
+    <row r="22" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="5"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="5"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="5"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="5"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+    </row>
+    <row r="23" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+    </row>
+    <row r="24" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+    </row>
+    <row r="25" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+    </row>
+    <row r="26" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+    </row>
+    <row r="27" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="D3"/>
-    <hyperlink r:id="rId2" ref="D4"/>
-    <hyperlink r:id="rId3" ref="D5"/>
-    <hyperlink r:id="rId4" ref="D6"/>
-    <hyperlink r:id="rId5" ref="D7"/>
-    <hyperlink r:id="rId6" ref="D8"/>
-    <hyperlink r:id="rId7" ref="D9"/>
-    <hyperlink r:id="rId8" ref="D10"/>
-    <hyperlink r:id="rId9" ref="D11"/>
-    <hyperlink r:id="rId10" ref="D12"/>
-    <hyperlink r:id="rId11" ref="D13"/>
-    <hyperlink r:id="rId12" ref="D14"/>
-    <hyperlink r:id="rId13" ref="D15"/>
-    <hyperlink r:id="rId14" ref="D16"/>
-    <hyperlink r:id="rId15" ref="D17"/>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
+    <hyperlink ref="D4" r:id="rId2" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
+    <hyperlink ref="D5" r:id="rId3" xr:uid="{00000000-0004-0000-0300-000002000000}"/>
+    <hyperlink ref="D6" r:id="rId4" xr:uid="{00000000-0004-0000-0300-000003000000}"/>
+    <hyperlink ref="D7" r:id="rId5" xr:uid="{00000000-0004-0000-0300-000004000000}"/>
+    <hyperlink ref="D8" r:id="rId6" xr:uid="{00000000-0004-0000-0300-000005000000}"/>
+    <hyperlink ref="D9" r:id="rId7" xr:uid="{00000000-0004-0000-0300-000006000000}"/>
+    <hyperlink ref="D10" r:id="rId8" xr:uid="{00000000-0004-0000-0300-000007000000}"/>
+    <hyperlink ref="D11" r:id="rId9" xr:uid="{00000000-0004-0000-0300-000008000000}"/>
+    <hyperlink ref="D12" r:id="rId10" xr:uid="{00000000-0004-0000-0300-000009000000}"/>
+    <hyperlink ref="D13" r:id="rId11" xr:uid="{00000000-0004-0000-0300-00000A000000}"/>
+    <hyperlink ref="D14" r:id="rId12" xr:uid="{00000000-0004-0000-0300-00000B000000}"/>
+    <hyperlink ref="D15" r:id="rId13" xr:uid="{00000000-0004-0000-0300-00000C000000}"/>
+    <hyperlink ref="D16" r:id="rId14" xr:uid="{00000000-0004-0000-0300-00000D000000}"/>
+    <hyperlink ref="D17" r:id="rId15" xr:uid="{00000000-0004-0000-0300-00000E000000}"/>
   </hyperlinks>
-  <drawing r:id="rId16"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:D32"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="62.5"/>
-    <col customWidth="1" min="2" max="2" width="20.13"/>
-    <col customWidth="1" min="3" max="3" width="19.5"/>
-    <col customWidth="1" min="4" max="4" width="25.25"/>
+    <col min="1" max="1" width="62.42578125" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" customWidth="1"/>
+    <col min="4" max="4" width="25.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.0" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="11" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+    </row>
+    <row r="2" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="s">
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+    </row>
+    <row r="4" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="s">
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="s">
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="s">
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="s">
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="s">
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+    </row>
+    <row r="9" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="s">
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="s">
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="s">
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="s">
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+    </row>
+    <row r="13" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="s">
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="s">
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+    </row>
+    <row r="15" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="s">
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+    </row>
+    <row r="16" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="s">
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+    </row>
+    <row r="17" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="s">
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+    </row>
+    <row r="18" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="s">
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+    </row>
+    <row r="19" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="s">
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+    </row>
+    <row r="20" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="s">
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+    </row>
+    <row r="21" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="s">
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+    </row>
+    <row r="22" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="s">
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+    </row>
+    <row r="23" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="s">
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+    </row>
+    <row r="24" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="s">
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+    </row>
+    <row r="25" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="s">
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+    </row>
+    <row r="26" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="s">
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+    </row>
+    <row r="27" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A27" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="s">
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+    </row>
+    <row r="28" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="4" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="s">
+    <row r="29" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="4" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="s">
+    <row r="30" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A30" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="4" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="s">
+    <row r="31" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A31" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="3" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="s">
+    <row r="32" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A32" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="4" t="s">
         <v>255</v>
       </c>
     </row>
@@ -3002,441 +2999,445 @@
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:D46"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="62.5"/>
-    <col customWidth="1" min="2" max="2" width="20.13"/>
-    <col customWidth="1" min="3" max="3" width="19.5"/>
-    <col customWidth="1" min="4" max="4" width="25.25"/>
+    <col min="1" max="1" width="62.42578125" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" customWidth="1"/>
+    <col min="4" max="4" width="25.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.0" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="11" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+    </row>
+    <row r="2" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="s">
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+    </row>
+    <row r="4" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="s">
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="s">
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="s">
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="s">
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>265</v>
       </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="s">
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+    </row>
+    <row r="9" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="s">
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="s">
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="s">
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="s">
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+    </row>
+    <row r="13" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="s">
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="s">
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+    </row>
+    <row r="15" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="s">
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+    </row>
+    <row r="16" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="s">
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+    </row>
+    <row r="17" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="s">
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+    </row>
+    <row r="18" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="s">
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+    </row>
+    <row r="19" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>271</v>
       </c>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="s">
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+    </row>
+    <row r="20" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="s">
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+    </row>
+    <row r="21" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="s">
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+    </row>
+    <row r="22" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="s">
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+    </row>
+    <row r="23" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="s">
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+    </row>
+    <row r="24" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="s">
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+    </row>
+    <row r="25" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="s">
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+    </row>
+    <row r="26" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="4" t="s">
         <v>281</v>
       </c>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="s">
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+    </row>
+    <row r="27" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A27" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="s">
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+    </row>
+    <row r="28" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="4" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="s">
+    <row r="29" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="4" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="s">
+    <row r="30" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A30" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="4" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="s">
+    <row r="31" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A31" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="4" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="s">
+    <row r="32" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A32" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="4" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="s">
+    <row r="33" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A33" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="4" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="s">
+    <row r="34" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A34" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="4" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="s">
+    <row r="35" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A35" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="4" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="s">
+    <row r="36" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A36" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="4" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="s">
+    <row r="37" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A37" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="4" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="s">
+    <row r="38" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A38" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="B38" s="4" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="s">
+    <row r="39" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A39" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="B39" s="4" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="s">
+    <row r="40" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A40" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="B40" s="4" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="s">
+    <row r="41" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A41" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="B41" s="4" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="s">
+    <row r="42" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A42" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="B42" s="4" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="s">
+    <row r="43" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A43" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="B43" s="4" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="s">
+    <row r="44" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A44" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B44" s="4" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="4" t="s">
+    <row r="45" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A45" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B45" s="4" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="s">
+    <row r="46" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A46" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B46" s="4" t="s">
         <v>301</v>
       </c>
     </row>
@@ -3444,6 +3445,6 @@
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>